<commit_message>
Added Diskann Age scripts
</commit_message>
<xml_diff>
--- a/ADF_SHIR_ProjectPlan.xlsx
+++ b/ADF_SHIR_ProjectPlan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Alok_Sharma/Documents/myrepo/diskann-age-demo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E6008A-4089-6A42-9EF6-8B220355AD40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25AE1DCF-CAB6-6D42-B9D9-960CAE4D0AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="272">
   <si>
     <t>Phase</t>
   </si>
@@ -947,7 +947,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -960,25 +960,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1335,512 +1320,512 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="13" t="s">
         <v>270</v>
       </c>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9" t="s">
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="H2" s="9"/>
+      <c r="H2" s="8"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="10"/>
-      <c r="B3" s="9" t="s">
+      <c r="A3" s="14"/>
+      <c r="B3" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="19"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9" t="s">
+      <c r="D3" s="14"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="H3" s="9"/>
+      <c r="H3" s="8"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="10"/>
-      <c r="B4" s="9" t="s">
+      <c r="A4" s="14"/>
+      <c r="B4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9" t="s">
+      <c r="D4" s="14"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="H4" s="9"/>
+      <c r="H4" s="8"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="10"/>
-      <c r="B5" s="9" t="s">
+      <c r="A5" s="14"/>
+      <c r="B5" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="19"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9" t="s">
+      <c r="D5" s="14"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="H5" s="9"/>
+      <c r="H5" s="8"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="10"/>
-      <c r="B6" s="9" t="s">
+      <c r="A6" s="14"/>
+      <c r="B6" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="19"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9" t="s">
+      <c r="D6" s="14"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="H6" s="9"/>
+      <c r="H6" s="8"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="10"/>
-      <c r="B7" s="9" t="s">
+      <c r="A7" s="14"/>
+      <c r="B7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="19"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9" t="s">
+      <c r="D7" s="14"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="8" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="10"/>
-      <c r="B8" s="9" t="s">
+      <c r="A8" s="14"/>
+      <c r="B8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="19"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9" t="s">
+      <c r="D8" s="14"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="8" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="10"/>
-      <c r="B9" s="9" t="s">
+      <c r="A9" s="14"/>
+      <c r="B9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="19"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="11" t="s">
+      <c r="D9" s="14"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H9" s="9"/>
+      <c r="H9" s="8"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="15" t="s">
         <v>270</v>
       </c>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="12"/>
-      <c r="B11" s="13" t="s">
+      <c r="A11" s="15"/>
+      <c r="B11" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="20"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13" t="s">
+      <c r="D11" s="15"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="H11" s="10" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="12"/>
-      <c r="B12" s="13" t="s">
+      <c r="A12" s="15"/>
+      <c r="B12" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="20"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13" t="s">
+      <c r="D12" s="15"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H12" s="13" t="s">
+      <c r="H12" s="10" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="12"/>
-      <c r="B13" s="13" t="s">
+      <c r="A13" s="15"/>
+      <c r="B13" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="20"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13" t="s">
+      <c r="D13" s="15"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H13" s="13" t="s">
+      <c r="H13" s="10" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="12"/>
-      <c r="B14" s="13" t="s">
+      <c r="A14" s="15"/>
+      <c r="B14" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="20"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13" t="s">
+      <c r="D14" s="15"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H14" s="13" t="s">
+      <c r="H14" s="10" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="12"/>
-      <c r="B15" s="13" t="s">
+      <c r="A15" s="15"/>
+      <c r="B15" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D15" s="20"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13" t="s">
+      <c r="D15" s="15"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H15" s="13" t="s">
+      <c r="H15" s="10" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="12"/>
-      <c r="B16" s="13" t="s">
+      <c r="A16" s="15"/>
+      <c r="B16" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="20"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13" t="s">
+      <c r="D16" s="15"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="H16" s="13" t="s">
+      <c r="H16" s="10" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="15" t="s">
+      <c r="B17" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C17" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="21" t="s">
+      <c r="D17" s="16" t="s">
         <v>270</v>
       </c>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="14"/>
-      <c r="B18" s="15" t="s">
+      <c r="A18" s="16"/>
+      <c r="B18" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="21"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15" t="s">
+      <c r="D18" s="16"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H18" s="15" t="s">
+      <c r="H18" s="11" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="14"/>
-      <c r="B19" s="15" t="s">
+      <c r="A19" s="16"/>
+      <c r="B19" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="D19" s="21"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15" t="s">
+      <c r="D19" s="16"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="H19" s="15" t="s">
+      <c r="H19" s="11" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="14"/>
-      <c r="B20" s="15" t="s">
+      <c r="A20" s="16"/>
+      <c r="B20" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="D20" s="21"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="15" t="s">
+      <c r="D20" s="16"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="H20" s="15" t="s">
+      <c r="H20" s="11" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="14"/>
-      <c r="B21" s="15" t="s">
+      <c r="A21" s="16"/>
+      <c r="B21" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="15" t="s">
+      <c r="C21" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="D21" s="21"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="15" t="s">
+      <c r="D21" s="16"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="H21" s="15" t="s">
+      <c r="H21" s="11" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D22" s="22" t="s">
+      <c r="D22" s="17" t="s">
         <v>270</v>
       </c>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17" t="s">
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="H22" s="17" t="s">
+      <c r="H22" s="12" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="16"/>
-      <c r="B23" s="17" t="s">
+      <c r="A23" s="17"/>
+      <c r="B23" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D23" s="22"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17" t="s">
+      <c r="D23" s="17"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="H23" s="17" t="s">
+      <c r="H23" s="12" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="16"/>
-      <c r="B24" s="17" t="s">
+      <c r="A24" s="17"/>
+      <c r="B24" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="C24" s="17" t="s">
+      <c r="C24" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D24" s="22"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="16"/>
-      <c r="B25" s="17" t="s">
+      <c r="A25" s="17"/>
+      <c r="B25" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="C25" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D25" s="22"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="16"/>
-      <c r="B26" s="17" t="s">
+      <c r="A26" s="17"/>
+      <c r="B26" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="17" t="s">
+      <c r="C26" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D26" s="22"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17" t="s">
+      <c r="D26" s="17"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="H26" s="17" t="s">
+      <c r="H26" s="12" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A27" s="16"/>
-      <c r="B27" s="17" t="s">
+      <c r="A27" s="17"/>
+      <c r="B27" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="C27" s="17" t="s">
+      <c r="C27" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D27" s="22"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="17" t="s">
+      <c r="D27" s="17"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="H27" s="17" t="s">
+      <c r="H27" s="12" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A28" s="16"/>
-      <c r="B28" s="17" t="s">
+      <c r="A28" s="17"/>
+      <c r="B28" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="C28" s="17" t="s">
+      <c r="C28" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D28" s="22"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="17" t="s">
+      <c r="D28" s="17"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="H28" s="17" t="s">
+      <c r="H28" s="12" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" s="16"/>
-      <c r="B29" s="17" t="s">
+      <c r="A29" s="17"/>
+      <c r="B29" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D29" s="22"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="17" t="s">
+      <c r="D29" s="17"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="H29" s="17" t="s">
+      <c r="H29" s="12" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" s="16"/>
-      <c r="B30" s="17" t="s">
+      <c r="A30" s="17"/>
+      <c r="B30" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="C30" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D30" s="22"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="17" t="s">
+      <c r="D30" s="17"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="H30" s="17" t="s">
+      <c r="H30" s="12" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1861,51 +1846,59 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="C1" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="C3" s="5"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="C4" s="5"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="5">
         <v>1</v>
       </c>
+      <c r="C5" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>